<commit_message>
ofav transcriptomics, aesthetic changes
</commit_message>
<xml_diff>
--- a/outputs/photosynthesis/coral_FvFm_GAMM_stats.xlsx
+++ b/outputs/photosynthesis/coral_FvFm_GAMM_stats.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Model fit" sheetId="1" r:id="rId1"/>
     <sheet name="Rho estimates" sheetId="2" r:id="rId2"/>
     <sheet name="Joint tests" sheetId="3" r:id="rId3"/>
-    <sheet name="Parametric coefficients" sheetId="4" r:id="rId4"/>
+    <sheet name="Effects vs overall mean" sheetId="4" r:id="rId4"/>
     <sheet name="Smooth significance" sheetId="5" r:id="rId5"/>
     <sheet name="k.check" sheetId="6" r:id="rId6"/>
     <sheet name="Estimated marginal means" sheetId="7" r:id="rId7"/>
@@ -888,7 +888,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:G81"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -904,20 +904,25 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>std_error</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>t_value</t>
+          <t>df</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>t_ratio</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>p_value</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>model</t>
         </is>
@@ -926,22 +931,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>(Intercept)</t>
+          <t>overall mean</t>
         </is>
       </c>
       <c r="B2">
-        <v>0.4386256879721936</v>
+        <v>0.4356588237227743</v>
       </c>
       <c r="C2">
-        <v>0.01162963068231404</v>
+        <v>0.004443022444785122</v>
       </c>
       <c r="D2">
-        <v>37.71621816325098</v>
-      </c>
-      <c r="E2">
-        <v>5.131663032553078E-86</v>
-      </c>
-      <c r="F2" t="inlineStr">
+        <v>175.2045442285989</v>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>ofav_control</t>
         </is>
@@ -950,22 +952,25 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>treatmentLC:siteRainbow</t>
+          <t>treatment CC</t>
         </is>
       </c>
       <c r="B3">
-        <v>0.05103480058539134</v>
+        <v>-0.009736001586646496</v>
       </c>
       <c r="C3">
-        <v>0.03899314648083595</v>
+        <v>0.006886396904334061</v>
       </c>
       <c r="D3">
-        <v>1.3088146300395</v>
+        <v>175.2045442285989</v>
       </c>
       <c r="E3">
-        <v>0.1923112665405252</v>
-      </c>
-      <c r="F3" t="inlineStr">
+        <v>-1.413801981195564</v>
+      </c>
+      <c r="F3">
+        <v>0.1591944326277489</v>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>ofav_control</t>
         </is>
@@ -974,22 +979,25 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>treatmentCH:siteRainbow</t>
+          <t>treatment LC</t>
         </is>
       </c>
       <c r="B4">
-        <v>-0.03156642279546758</v>
+        <v>-0.04015305218057764</v>
       </c>
       <c r="C4">
-        <v>0.02678917137592421</v>
+        <v>0.008297200450431653</v>
       </c>
       <c r="D4">
-        <v>-1.178327703851145</v>
+        <v>175.2045442285989</v>
       </c>
       <c r="E4">
-        <v>0.2402638944666043</v>
-      </c>
-      <c r="F4" t="inlineStr">
+        <v>-4.839349419175321</v>
+      </c>
+      <c r="F4">
+        <v>2.844113068834794E-06</v>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>ofav_control</t>
         </is>
@@ -998,22 +1006,25 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>treatmentLH:siteRainbow</t>
+          <t>treatment CH</t>
         </is>
       </c>
       <c r="B5">
-        <v>-0.03836506878535723</v>
+        <v>0.009141159838930216</v>
       </c>
       <c r="C5">
-        <v>0.03740091221718866</v>
+        <v>0.006159902588585336</v>
       </c>
       <c r="D5">
-        <v>-1.025778958613888</v>
+        <v>175.2045442285989</v>
       </c>
       <c r="E5">
-        <v>0.3064099342031821</v>
-      </c>
-      <c r="F5" t="inlineStr">
+        <v>1.483977986254089</v>
+      </c>
+      <c r="F5">
+        <v>0.1396115357719038</v>
+      </c>
+      <c r="G5" t="inlineStr">
         <is>
           <t>ofav_control</t>
         </is>
@@ -1022,22 +1033,25 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>treatmentLC:siteStar</t>
+          <t>treatment LH</t>
         </is>
       </c>
       <c r="B6">
-        <v>0.02503130922524261</v>
+        <v>0.04074789392829394</v>
       </c>
       <c r="C6">
-        <v>0.03119451718466873</v>
+        <v>0.009083726044889214</v>
       </c>
       <c r="D6">
-        <v>0.8024265635226703</v>
+        <v>175.2045442285989</v>
       </c>
       <c r="E6">
-        <v>0.4233933524524296</v>
-      </c>
-      <c r="F6" t="inlineStr">
+        <v>4.485812730032734</v>
+      </c>
+      <c r="F6">
+        <v>1.310841084099791E-05</v>
+      </c>
+      <c r="G6" t="inlineStr">
         <is>
           <t>ofav_control</t>
         </is>
@@ -1046,22 +1060,25 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>treatmentCH:siteStar</t>
+          <t>site Emerald</t>
         </is>
       </c>
       <c r="B7">
-        <v>-0.01268907931033241</v>
+        <v>-0.05638290572290167</v>
       </c>
       <c r="C7">
-        <v>0.02678917137592421</v>
+        <v>0.007073789604240152</v>
       </c>
       <c r="D7">
-        <v>-0.4736644942193419</v>
+        <v>175.2045442285989</v>
       </c>
       <c r="E7">
-        <v>0.6363288595428018</v>
-      </c>
-      <c r="F7" t="inlineStr">
+        <v>-7.970678925636235</v>
+      </c>
+      <c r="F7">
+        <v>1.945860798849331E-13</v>
+      </c>
+      <c r="G7" t="inlineStr">
         <is>
           <t>ofav_control</t>
         </is>
@@ -1070,22 +1087,25 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>treatmentLH:siteStar</t>
+          <t>site Rainbow</t>
         </is>
       </c>
       <c r="B8">
-        <v>-0.01551799636626711</v>
+        <v>-0.02638840336268705</v>
       </c>
       <c r="C8">
-        <v>0.03740091221718864</v>
+        <v>0.008888301942539239</v>
       </c>
       <c r="D8">
-        <v>-0.4149095689472349</v>
+        <v>175.2045442285989</v>
       </c>
       <c r="E8">
-        <v>0.6787157146962113</v>
-      </c>
-      <c r="F8" t="inlineStr">
+        <v>-2.968891418550113</v>
+      </c>
+      <c r="F8">
+        <v>0.003407430084079613</v>
+      </c>
+      <c r="G8" t="inlineStr">
         <is>
           <t>ofav_control</t>
         </is>
@@ -1094,22 +1114,25 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>treatmentLC:siteMacN</t>
+          <t>site Star</t>
         </is>
       </c>
       <c r="B9">
-        <v>0.01990324763414215</v>
+        <v>0.0408901940722853</v>
       </c>
       <c r="C9">
-        <v>0.03119451718466874</v>
+        <v>0.007846489347296931</v>
       </c>
       <c r="D9">
-        <v>0.6380367266566979</v>
+        <v>175.2045442285989</v>
       </c>
       <c r="E9">
-        <v>0.5242828059518212</v>
-      </c>
-      <c r="F9" t="inlineStr">
+        <v>5.211272489189287</v>
+      </c>
+      <c r="F9">
+        <v>5.231526800093123E-07</v>
+      </c>
+      <c r="G9" t="inlineStr">
         <is>
           <t>ofav_control</t>
         </is>
@@ -1118,22 +1141,25 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>treatmentCH:siteMacN</t>
+          <t>site MacN</t>
         </is>
       </c>
       <c r="B10">
-        <v>-0.02216949829613561</v>
+        <v>0.04188111501330342</v>
       </c>
       <c r="C10">
-        <v>0.02514982378765276</v>
+        <v>0.006732068490519134</v>
       </c>
       <c r="D10">
-        <v>-0.8814971621001839</v>
+        <v>175.2045442285989</v>
       </c>
       <c r="E10">
-        <v>0.3792564790982089</v>
-      </c>
-      <c r="F10" t="inlineStr">
+        <v>6.221136203870352</v>
+      </c>
+      <c r="F10">
+        <v>3.523502928324561E-09</v>
+      </c>
+      <c r="G10" t="inlineStr">
         <is>
           <t>ofav_control</t>
         </is>
@@ -1142,22 +1168,25 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>treatmentLH:siteMacN</t>
+          <t>treatment x site CC : Emerald</t>
         </is>
       </c>
       <c r="B11">
-        <v>-0.0231311198819238</v>
+        <v>-0.002966864249419228</v>
       </c>
       <c r="C11">
-        <v>0.02917979891271558</v>
+        <v>0.01097927152591337</v>
       </c>
       <c r="D11">
-        <v>-0.7927100509196463</v>
+        <v>175.2045442285989</v>
       </c>
       <c r="E11">
-        <v>0.4290188727792749</v>
-      </c>
-      <c r="F11" t="inlineStr">
+        <v>-0.2702241439622666</v>
+      </c>
+      <c r="F11">
+        <v>0.787305858791389</v>
+      </c>
+      <c r="G11" t="inlineStr">
         <is>
           <t>ofav_control</t>
         </is>
@@ -1166,430 +1195,1870 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>(Intercept)</t>
+          <t>treatment x site LC : Emerald</t>
         </is>
       </c>
       <c r="B12">
-        <v>0.3945470664665202</v>
+        <v>-0.02695920361061325</v>
       </c>
       <c r="C12">
-        <v>0.01389093318102155</v>
+        <v>0.01367716226636776</v>
       </c>
       <c r="D12">
-        <v>28.40320814483285</v>
+        <v>175.2045442285989</v>
       </c>
       <c r="E12">
-        <v>3.828954088859774E-99</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>ofav_heat</t>
+        <v>-1.971110898998846</v>
+      </c>
+      <c r="F12">
+        <v>0.05028606800358819</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>ofav_control</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>treatmentLH:siteRainbow</t>
+          <t>treatment x site CH : Emerald</t>
         </is>
       </c>
       <c r="B13">
-        <v>0.02778022203094027</v>
+        <v>0.01363938585106467</v>
       </c>
       <c r="C13">
-        <v>0.04666346702117233</v>
+        <v>0.01011428779351373</v>
       </c>
       <c r="D13">
-        <v>0.5953312902861617</v>
+        <v>175.2045442285989</v>
       </c>
       <c r="E13">
-        <v>0.5519482861519334</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>ofav_heat</t>
+        <v>1.348526572460355</v>
+      </c>
+      <c r="F13">
+        <v>0.1792296710329647</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>ofav_control</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>treatmentLH:siteStar</t>
+          <t>treatment x site LH : Emerald</t>
         </is>
       </c>
       <c r="B14">
-        <v>-0.03637784107739722</v>
+        <v>0.0162866820089678</v>
       </c>
       <c r="C14">
-        <v>0.03866704233954938</v>
+        <v>0.01303685280637928</v>
       </c>
       <c r="D14">
-        <v>-0.9407970942786404</v>
+        <v>175.2045442285989</v>
       </c>
       <c r="E14">
-        <v>0.3473590868962794</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>ofav_heat</t>
+        <v>1.249280194449867</v>
+      </c>
+      <c r="F14">
+        <v>0.2132290393411336</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>ofav_control</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>treatmentLH:siteMacN</t>
+          <t>treatment x site CC : Rainbow</t>
         </is>
       </c>
       <c r="B15">
-        <v>-0.00588250088840088</v>
+        <v>0.001757308499439142</v>
       </c>
       <c r="C15">
-        <v>0.03690979149786645</v>
+        <v>0.01281630935852498</v>
       </c>
       <c r="D15">
-        <v>-0.1593750777145657</v>
+        <v>175.2045442285989</v>
       </c>
       <c r="E15">
-        <v>0.8734513259167644</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>ofav_heat</t>
+        <v>0.1371150188622936</v>
+      </c>
+      <c r="F15">
+        <v>0.8910973194922308</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>ofav_control</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>(Intercept)</t>
+          <t>treatment x site LC : Rainbow</t>
         </is>
       </c>
       <c r="B16">
-        <v>0.3138184996420411</v>
+        <v>0.02879976972363645</v>
       </c>
       <c r="C16">
-        <v>0.01285164456162865</v>
+        <v>0.01751574787492767</v>
       </c>
       <c r="D16">
-        <v>24.41854800272127</v>
+        <v>175.2045442285989</v>
       </c>
       <c r="E16">
-        <v>7.472337606185724E-73</v>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>ssid_control</t>
+        <v>1.64422152735259</v>
+      </c>
+      <c r="F16">
+        <v>0.1019235878615577</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>ofav_control</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>treatmentLC:siteRainbow</t>
+          <t>treatment x site CH : Rainbow</t>
         </is>
       </c>
       <c r="B17">
-        <v>-0.0135905832761481</v>
+        <v>-0.01320286419554454</v>
       </c>
       <c r="C17">
-        <v>0.03210613509143157</v>
+        <v>0.01143711262421352</v>
       </c>
       <c r="D17">
-        <v>-0.42330175330805</v>
+        <v>175.2045442285989</v>
       </c>
       <c r="E17">
-        <v>0.672382977309413</v>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>ssid_control</t>
+        <v>-1.15438787999628</v>
+      </c>
+      <c r="F17">
+        <v>0.2499133217254166</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>ofav_control</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>treatmentCH:siteRainbow</t>
+          <t>treatment x site LH : Rainbow</t>
         </is>
       </c>
       <c r="B18">
-        <v>0.04963062453130374</v>
+        <v>-0.01735421402753106</v>
       </c>
       <c r="C18">
-        <v>0.03210613509143156</v>
+        <v>0.01789149229388642</v>
       </c>
       <c r="D18">
-        <v>1.545829929076362</v>
+        <v>175.2045442285989</v>
       </c>
       <c r="E18">
-        <v>0.1232157107501538</v>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>ssid_control</t>
+        <v>-0.9699701814957632</v>
+      </c>
+      <c r="F18">
+        <v>0.3333984872000813</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>ofav_control</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>treatmentLH:siteRainbow</t>
+          <t>treatment x site CC : Star</t>
         </is>
       </c>
       <c r="B19">
-        <v>0.0370205683824967</v>
+        <v>-0.002172922636580001</v>
       </c>
       <c r="C19">
-        <v>0.03210613509143152</v>
+        <v>0.01213064503676786</v>
       </c>
       <c r="D19">
-        <v>1.15306835522463</v>
+        <v>175.2045442285989</v>
       </c>
       <c r="E19">
-        <v>0.2498140208310467</v>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>ssid_control</t>
+        <v>-0.1791267183232133</v>
+      </c>
+      <c r="F19">
+        <v>0.8580451812037124</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>ofav_control</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>treatmentLC:siteStar</t>
+          <t>treatment x site LC : Star</t>
         </is>
       </c>
       <c r="B20">
-        <v>0.01730873497980174</v>
+        <v>-0.001133952772531416</v>
       </c>
       <c r="C20">
-        <v>0.03210613509143156</v>
+        <v>0.01236342567939183</v>
       </c>
       <c r="D20">
-        <v>0.5391098906956593</v>
+        <v>175.2045442285989</v>
       </c>
       <c r="E20">
-        <v>0.5902168964895658</v>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>ssid_control</t>
+        <v>-0.09171833130534064</v>
+      </c>
+      <c r="F20">
+        <v>0.9270266149050699</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>ofav_control</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>treatmentCH:siteStar</t>
+          <t>treatment x site CH : Star</t>
         </is>
       </c>
       <c r="B21">
-        <v>0.0686361477464959</v>
+        <v>0.00174424815357149</v>
       </c>
       <c r="C21">
-        <v>0.03210613509143164</v>
+        <v>0.01066312846277256</v>
       </c>
       <c r="D21">
-        <v>2.13778916556086</v>
+        <v>175.2045442285989</v>
       </c>
       <c r="E21">
-        <v>0.03335407221107774</v>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>ssid_control</t>
+        <v>0.163577524144163</v>
+      </c>
+      <c r="F21">
+        <v>0.8702522770598331</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>ofav_control</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>treatmentLH:siteStar</t>
+          <t>treatment x site LH : Star</t>
         </is>
       </c>
       <c r="B22">
-        <v>0.04411885837877381</v>
+        <v>0.001562627255539926</v>
       </c>
       <c r="C22">
-        <v>0.03210613509143161</v>
+        <v>0.01740690265201833</v>
       </c>
       <c r="D22">
-        <v>1.37415662935238</v>
+        <v>175.2045442285989</v>
       </c>
       <c r="E22">
-        <v>0.1704342312671515</v>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>ssid_control</t>
+        <v>0.08977055176204705</v>
+      </c>
+      <c r="F22">
+        <v>0.928572089342566</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>ofav_control</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>treatmentLC:siteMacN</t>
+          <t>treatment x site CC : MacN</t>
         </is>
       </c>
       <c r="B23">
-        <v>-0.006843576505077798</v>
+        <v>0.003382478386560086</v>
       </c>
       <c r="C23">
-        <v>0.03309424655308052</v>
+        <v>0.01076954069690552</v>
       </c>
       <c r="D23">
-        <v>-0.2067905215518731</v>
+        <v>175.2045442285989</v>
       </c>
       <c r="E23">
-        <v>0.8363158515220516</v>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>ssid_control</t>
+        <v>0.3140782398948542</v>
+      </c>
+      <c r="F23">
+        <v>0.7538352726621881</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>ofav_control</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>treatmentCH:siteMacN</t>
+          <t>treatment x site LC : MacN</t>
         </is>
       </c>
       <c r="B24">
-        <v>0.0509272468954484</v>
+        <v>-0.0007066133404917858</v>
       </c>
       <c r="C24">
-        <v>0.03309424655308055</v>
+        <v>0.0123326421254169</v>
       </c>
       <c r="D24">
-        <v>1.538855003505371</v>
+        <v>175.2045442285989</v>
       </c>
       <c r="E24">
-        <v>0.124909604573518</v>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>ssid_control</t>
+        <v>-0.05729618465417841</v>
+      </c>
+      <c r="F24">
+        <v>0.9543745512840482</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>ofav_control</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>treatmentLH:siteMacN</t>
+          <t>treatment x site CH : MacN</t>
         </is>
       </c>
       <c r="B25">
-        <v>0.01794852772641631</v>
+        <v>-0.002180769809091622</v>
       </c>
       <c r="C25">
-        <v>0.03309424655308054</v>
+        <v>0.009573690994736012</v>
       </c>
       <c r="D25">
-        <v>0.5423458635817044</v>
+        <v>175.2045442285989</v>
       </c>
       <c r="E25">
-        <v>0.587988958188609</v>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>ssid_control</t>
+        <v>-0.2277877790593716</v>
+      </c>
+      <c r="F25">
+        <v>0.820076837028819</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>ofav_control</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>(Intercept)</t>
+          <t>treatment x site LH : MacN</t>
         </is>
       </c>
       <c r="B26">
-        <v>0.3205614863572391</v>
+        <v>-0.0004950952369766819</v>
       </c>
       <c r="C26">
-        <v>0.009399211856398094</v>
+        <v>0.01286072061269397</v>
       </c>
       <c r="D26">
-        <v>34.10514533077911</v>
+        <v>175.2045442285989</v>
       </c>
       <c r="E26">
-        <v>2.673552169490497E-126</v>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>ssid_heat</t>
+        <v>-0.03849669484989869</v>
+      </c>
+      <c r="F26">
+        <v>0.9693354962098961</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>ofav_control</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>treatmentLH:siteRainbow</t>
+          <t>overall mean</t>
         </is>
       </c>
       <c r="B27">
-        <v>-0.02388828650690011</v>
+        <v>0.3719293947695835</v>
       </c>
       <c r="C27">
-        <v>0.02660351065239026</v>
+        <v>0.007620731627183546</v>
       </c>
       <c r="D27">
-        <v>-0.8979373744703051</v>
-      </c>
-      <c r="E27">
-        <v>0.3697038561709641</v>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>ssid_heat</t>
+        <v>412.7735348871453</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>ofav_heat</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>treatmentLH:siteStar</t>
+          <t>treatment CH</t>
         </is>
       </c>
       <c r="B28">
-        <v>-0.02842690840831184</v>
+        <v>0.007106843717662075</v>
       </c>
       <c r="C28">
-        <v>0.02613019749612858</v>
+        <v>0.007631402060364536</v>
       </c>
       <c r="D28">
-        <v>-1.087894892969084</v>
+        <v>412.7735348871453</v>
       </c>
       <c r="E28">
-        <v>0.2772295879043122</v>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>ssid_heat</t>
+        <v>0.9312631756847307</v>
+      </c>
+      <c r="F28">
+        <v>0.3522617877451257</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>ofav_heat</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>treatmentLH:siteMacN</t>
+          <t>treatment LH</t>
         </is>
       </c>
       <c r="B29">
-        <v>-0.03739645439423202</v>
+        <v>-0.007106843717662075</v>
       </c>
       <c r="C29">
-        <v>0.02643497420496783</v>
+        <v>0.007631402060364536</v>
       </c>
       <c r="D29">
-        <v>-1.414658251764219</v>
+        <v>412.7735348871453</v>
       </c>
       <c r="E29">
-        <v>0.1578671151072505</v>
-      </c>
-      <c r="F29" t="inlineStr">
+        <v>-0.9312631756847307</v>
+      </c>
+      <c r="F29">
+        <v>0.3522617877451257</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>ofav_heat</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>site Emerald</t>
+        </is>
+      </c>
+      <c r="B30">
+        <v>-0.04042730096006027</v>
+      </c>
+      <c r="C30">
+        <v>0.01238871230368095</v>
+      </c>
+      <c r="D30">
+        <v>412.7735348871453</v>
+      </c>
+      <c r="E30">
+        <v>-3.26323672461491</v>
+      </c>
+      <c r="F30">
+        <v>0.00119311679529951</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>ofav_heat</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>site Rainbow</t>
+        </is>
+      </c>
+      <c r="B31">
+        <v>-0.02205637281695993</v>
+      </c>
+      <c r="C31">
+        <v>0.01529855369826901</v>
+      </c>
+      <c r="D31">
+        <v>412.7735348871453</v>
+      </c>
+      <c r="E31">
+        <v>-1.441729280556472</v>
+      </c>
+      <c r="F31">
+        <v>0.1501369990154243</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>ofav_heat</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>site Star</t>
+        </is>
+      </c>
+      <c r="B32">
+        <v>0.02449281209745503</v>
+      </c>
+      <c r="C32">
+        <v>0.01207732992163291</v>
+      </c>
+      <c r="D32">
+        <v>412.7735348871453</v>
+      </c>
+      <c r="E32">
+        <v>2.02799892495969</v>
+      </c>
+      <c r="F32">
+        <v>0.04320213056575246</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>ofav_heat</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>site MacN</t>
+        </is>
+      </c>
+      <c r="B33">
+        <v>0.03799086167956518</v>
+      </c>
+      <c r="C33">
+        <v>0.01143407299573432</v>
+      </c>
+      <c r="D33">
+        <v>412.7735348871453</v>
+      </c>
+      <c r="E33">
+        <v>3.322600939642272</v>
+      </c>
+      <c r="F33">
+        <v>0.0009713117844537503</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>ofav_heat</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>treatment x site CH : Emerald</t>
+        </is>
+      </c>
+      <c r="B34">
+        <v>-0.001810014991857307</v>
+      </c>
+      <c r="C34">
+        <v>0.01228241145547157</v>
+      </c>
+      <c r="D34">
+        <v>412.7735348871453</v>
+      </c>
+      <c r="E34">
+        <v>-0.1473664189169449</v>
+      </c>
+      <c r="F34">
+        <v>0.8829147627075981</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>ofav_heat</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>treatment x site LH : Emerald</t>
+        </is>
+      </c>
+      <c r="B35">
+        <v>0.001810014991857307</v>
+      </c>
+      <c r="C35">
+        <v>0.01228241145547157</v>
+      </c>
+      <c r="D35">
+        <v>412.7735348871453</v>
+      </c>
+      <c r="E35">
+        <v>0.1473664189169449</v>
+      </c>
+      <c r="F35">
+        <v>0.8829147627075981</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>ofav_heat</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>treatment x site CH : Rainbow</t>
+        </is>
+      </c>
+      <c r="B36">
+        <v>-0.01570012600732737</v>
+      </c>
+      <c r="C36">
+        <v>0.01518773985784276</v>
+      </c>
+      <c r="D36">
+        <v>412.7735348871453</v>
+      </c>
+      <c r="E36">
+        <v>-1.033736826827464</v>
+      </c>
+      <c r="F36">
+        <v>0.3018644722364796</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>ofav_heat</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>treatment x site LH : Rainbow</t>
+        </is>
+      </c>
+      <c r="B37">
+        <v>0.01570012600732737</v>
+      </c>
+      <c r="C37">
+        <v>0.01518773985784276</v>
+      </c>
+      <c r="D37">
+        <v>412.7735348871453</v>
+      </c>
+      <c r="E37">
+        <v>1.033736826827464</v>
+      </c>
+      <c r="F37">
+        <v>0.3018644722364796</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>ofav_heat</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>treatment x site CH : Star</t>
+        </is>
+      </c>
+      <c r="B38">
+        <v>0.01637890554684138</v>
+      </c>
+      <c r="C38">
+        <v>0.01205149547126986</v>
+      </c>
+      <c r="D38">
+        <v>412.7735348871453</v>
+      </c>
+      <c r="E38">
+        <v>1.359076604715808</v>
+      </c>
+      <c r="F38">
+        <v>0.1748644072510913</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>ofav_heat</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>treatment x site LH : Star</t>
+        </is>
+      </c>
+      <c r="B39">
+        <v>-0.01637890554684138</v>
+      </c>
+      <c r="C39">
+        <v>0.01205149547126986</v>
+      </c>
+      <c r="D39">
+        <v>412.7735348871453</v>
+      </c>
+      <c r="E39">
+        <v>-1.359076604715808</v>
+      </c>
+      <c r="F39">
+        <v>0.1748644072510913</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>ofav_heat</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>treatment x site CH : MacN</t>
+        </is>
+      </c>
+      <c r="B40">
+        <v>0.001131235452343272</v>
+      </c>
+      <c r="C40">
+        <v>0.01133771871427797</v>
+      </c>
+      <c r="D40">
+        <v>412.7735348871453</v>
+      </c>
+      <c r="E40">
+        <v>0.09977628488160228</v>
+      </c>
+      <c r="F40">
+        <v>0.9205703758899153</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>ofav_heat</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>treatment x site LH : MacN</t>
+        </is>
+      </c>
+      <c r="B41">
+        <v>-0.001131235452343272</v>
+      </c>
+      <c r="C41">
+        <v>0.01133771871427797</v>
+      </c>
+      <c r="D41">
+        <v>412.7735348871453</v>
+      </c>
+      <c r="E41">
+        <v>-0.09977628488160228</v>
+      </c>
+      <c r="F41">
+        <v>0.9205703758899153</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>ofav_heat</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>overall mean</t>
+        </is>
+      </c>
+      <c r="B42">
+        <v>0.33039078394576</v>
+      </c>
+      <c r="C42">
+        <v>0.004053770017972506</v>
+      </c>
+      <c r="D42">
+        <v>295.551040775367</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>ssid_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>treatment CC</t>
+        </is>
+      </c>
+      <c r="B43">
+        <v>0.05350051621656567</v>
+      </c>
+      <c r="C43">
+        <v>0.007128168673016529</v>
+      </c>
+      <c r="D43">
+        <v>295.551040775367</v>
+      </c>
+      <c r="E43">
+        <v>7.505506487113624</v>
+      </c>
+      <c r="F43">
+        <v>7.248968391100128E-13</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>ssid_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>treatment LC</t>
+        </is>
+      </c>
+      <c r="B44">
+        <v>0.02008407258272527</v>
+      </c>
+      <c r="C44">
+        <v>0.006984747891246344</v>
+      </c>
+      <c r="D44">
+        <v>295.551040775367</v>
+      </c>
+      <c r="E44">
+        <v>2.87541839668912</v>
+      </c>
+      <c r="F44">
+        <v>0.004328155502998678</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>ssid_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>treatment CH</t>
+        </is>
+      </c>
+      <c r="B45">
+        <v>-0.04062291823915393</v>
+      </c>
+      <c r="C45">
+        <v>0.006985151465669926</v>
+      </c>
+      <c r="D45">
+        <v>295.551040775367</v>
+      </c>
+      <c r="E45">
+        <v>-5.815610218161233</v>
+      </c>
+      <c r="F45">
+        <v>1.566899238762987E-08</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>ssid_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>treatment LH</t>
+        </is>
+      </c>
+      <c r="B46">
+        <v>-0.03296167056013703</v>
+      </c>
+      <c r="C46">
+        <v>0.006985078804288372</v>
+      </c>
+      <c r="D46">
+        <v>295.551040775367</v>
+      </c>
+      <c r="E46">
+        <v>-4.718868817900918</v>
+      </c>
+      <c r="F46">
+        <v>3.664707731085024E-06</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>ssid_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>site Emerald</t>
+        </is>
+      </c>
+      <c r="B47">
+        <v>0.002007308538242901</v>
+      </c>
+      <c r="C47">
+        <v>0.006984616628874524</v>
+      </c>
+      <c r="D47">
+        <v>295.551040775367</v>
+      </c>
+      <c r="E47">
+        <v>0.2873899377590251</v>
+      </c>
+      <c r="F47">
+        <v>0.7740151619469204</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>ssid_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>site Rainbow</t>
+        </is>
+      </c>
+      <c r="B48">
+        <v>-0.01225241774208586</v>
+      </c>
+      <c r="C48">
+        <v>0.006984162182690221</v>
+      </c>
+      <c r="D48">
+        <v>295.551040775367</v>
+      </c>
+      <c r="E48">
+        <v>-1.754314608050291</v>
+      </c>
+      <c r="F48">
+        <v>0.08041295627102457</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>ssid_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>site Star</t>
+        </is>
+      </c>
+      <c r="B49">
+        <v>0.01175297809753159</v>
+      </c>
+      <c r="C49">
+        <v>0.00698260637866632</v>
+      </c>
+      <c r="D49">
+        <v>295.551040775367</v>
+      </c>
+      <c r="E49">
+        <v>1.683179239981219</v>
+      </c>
+      <c r="F49">
+        <v>0.09339635142248127</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>ssid_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>site MacN</t>
+        </is>
+      </c>
+      <c r="B50">
+        <v>-0.001507868893688637</v>
+      </c>
+      <c r="C50">
+        <v>0.007127627580926786</v>
+      </c>
+      <c r="D50">
+        <v>295.551040775367</v>
+      </c>
+      <c r="E50">
+        <v>-0.21155270481915</v>
+      </c>
+      <c r="F50">
+        <v>0.8326018149063582</v>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>ssid_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>treatment x site CC : Emerald</t>
+        </is>
+      </c>
+      <c r="B51">
+        <v>0.01657228430371942</v>
+      </c>
+      <c r="C51">
+        <v>0.0121334970191632</v>
+      </c>
+      <c r="D51">
+        <v>295.551040775367</v>
+      </c>
+      <c r="E51">
+        <v>1.365829181607394</v>
+      </c>
+      <c r="F51">
+        <v>0.173031042054588</v>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>ssid_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>treatment x site LC : Emerald</t>
+        </is>
+      </c>
+      <c r="B52">
+        <v>0.01735364050407546</v>
+      </c>
+      <c r="C52">
+        <v>0.01205024734295223</v>
+      </c>
+      <c r="D52">
+        <v>295.551040775367</v>
+      </c>
+      <c r="E52">
+        <v>1.440106581233372</v>
+      </c>
+      <c r="F52">
+        <v>0.150895662601481</v>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>ssid_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>treatment x site CH : Emerald</t>
+        </is>
+      </c>
+      <c r="B53">
+        <v>-0.02572622048959259</v>
+      </c>
+      <c r="C53">
+        <v>0.01205024734295226</v>
+      </c>
+      <c r="D53">
+        <v>295.551040775367</v>
+      </c>
+      <c r="E53">
+        <v>-2.134912235194816</v>
+      </c>
+      <c r="F53">
+        <v>0.03359049559057953</v>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>ssid_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>treatment x site LH : Emerald</t>
+        </is>
+      </c>
+      <c r="B54">
+        <v>-0.008199704318202284</v>
+      </c>
+      <c r="C54">
+        <v>0.01205024734295224</v>
+      </c>
+      <c r="D54">
+        <v>295.551040775367</v>
+      </c>
+      <c r="E54">
+        <v>-0.6804594200299134</v>
+      </c>
+      <c r="F54">
+        <v>0.496746309202207</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>ssid_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>treatment x site CC : Rainbow</t>
+        </is>
+      </c>
+      <c r="B55">
+        <v>-0.001692868105693667</v>
+      </c>
+      <c r="C55">
+        <v>0.01213349701916314</v>
+      </c>
+      <c r="D55">
+        <v>295.551040775367</v>
+      </c>
+      <c r="E55">
+        <v>-0.1395202144130437</v>
+      </c>
+      <c r="F55">
+        <v>0.8891341095908338</v>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>ssid_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>treatment x site LC : Rainbow</t>
+        </is>
+      </c>
+      <c r="B56">
+        <v>-0.01450209518148572</v>
+      </c>
+      <c r="C56">
+        <v>0.01205024734295223</v>
+      </c>
+      <c r="D56">
+        <v>295.551040775367</v>
+      </c>
+      <c r="E56">
+        <v>-1.203468673194289</v>
+      </c>
+      <c r="F56">
+        <v>0.2297580717222444</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>ssid_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>treatment x site CH : Rainbow</t>
+        </is>
+      </c>
+      <c r="B57">
+        <v>0.005639251632298061</v>
+      </c>
+      <c r="C57">
+        <v>0.01205024734295222</v>
+      </c>
+      <c r="D57">
+        <v>295.551040775367</v>
+      </c>
+      <c r="E57">
+        <v>0.4679780814288652</v>
+      </c>
+      <c r="F57">
+        <v>0.6401451699196075</v>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>ssid_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>treatment x site LH : Rainbow</t>
+        </is>
+      </c>
+      <c r="B58">
+        <v>0.01055571165488133</v>
+      </c>
+      <c r="C58">
+        <v>0.01205024734295222</v>
+      </c>
+      <c r="D58">
+        <v>295.551040775367</v>
+      </c>
+      <c r="E58">
+        <v>0.8759746878602461</v>
+      </c>
+      <c r="F58">
+        <v>0.3817551719459478</v>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>ssid_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>treatment x site CC : Star</t>
+        </is>
+      </c>
+      <c r="B59">
+        <v>-0.01594365097254844</v>
+      </c>
+      <c r="C59">
+        <v>0.01213349701916316</v>
+      </c>
+      <c r="D59">
+        <v>295.551040775367</v>
+      </c>
+      <c r="E59">
+        <v>-1.31401944116916</v>
+      </c>
+      <c r="F59">
+        <v>0.1898586243441945</v>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>ssid_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>treatment x site LC : Star</t>
+        </is>
+      </c>
+      <c r="B60">
+        <v>0.002146440207609335</v>
+      </c>
+      <c r="C60">
+        <v>0.01205024734295223</v>
+      </c>
+      <c r="D60">
+        <v>295.551040775367</v>
+      </c>
+      <c r="E60">
+        <v>0.178124161813551</v>
+      </c>
+      <c r="F60">
+        <v>0.8587474944770664</v>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>ssid_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>treatment x site CH : Star</t>
+        </is>
+      </c>
+      <c r="B61">
+        <v>0.01039399198063545</v>
+      </c>
+      <c r="C61">
+        <v>0.01205024734295225</v>
+      </c>
+      <c r="D61">
+        <v>295.551040775367</v>
+      </c>
+      <c r="E61">
+        <v>0.8625542434790362</v>
+      </c>
+      <c r="F61">
+        <v>0.3890819459952305</v>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>ssid_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>treatment x site LH : Star</t>
+        </is>
+      </c>
+      <c r="B62">
+        <v>0.003403218784303663</v>
+      </c>
+      <c r="C62">
+        <v>0.01205024734295224</v>
+      </c>
+      <c r="D62">
+        <v>295.551040775367</v>
+      </c>
+      <c r="E62">
+        <v>0.2824189983365017</v>
+      </c>
+      <c r="F62">
+        <v>0.7778199247702895</v>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>ssid_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>treatment x site CC : MacN</t>
+        </is>
+      </c>
+      <c r="B63">
+        <v>0.001064234774522691</v>
+      </c>
+      <c r="C63">
+        <v>0.01285851274072789</v>
+      </c>
+      <c r="D63">
+        <v>295.551040775367</v>
+      </c>
+      <c r="E63">
+        <v>0.08276499747531824</v>
+      </c>
+      <c r="F63">
+        <v>0.9340944271399774</v>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>ssid_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>treatment x site LC : MacN</t>
+        </is>
+      </c>
+      <c r="B64">
+        <v>-0.004997985530199068</v>
+      </c>
+      <c r="C64">
+        <v>0.01213349701916313</v>
+      </c>
+      <c r="D64">
+        <v>295.551040775367</v>
+      </c>
+      <c r="E64">
+        <v>-0.4119163273626276</v>
+      </c>
+      <c r="F64">
+        <v>0.680699336247149</v>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>ssid_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>treatment x site CH : MacN</t>
+        </is>
+      </c>
+      <c r="B65">
+        <v>0.009692976876659086</v>
+      </c>
+      <c r="C65">
+        <v>0.01213349701916315</v>
+      </c>
+      <c r="D65">
+        <v>295.551040775367</v>
+      </c>
+      <c r="E65">
+        <v>0.7988609434980201</v>
+      </c>
+      <c r="F65">
+        <v>0.4250125410162635</v>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>ssid_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>treatment x site LH : MacN</t>
+        </is>
+      </c>
+      <c r="B66">
+        <v>-0.005759226120982705</v>
+      </c>
+      <c r="C66">
+        <v>0.01213349701916314</v>
+      </c>
+      <c r="D66">
+        <v>295.551040775367</v>
+      </c>
+      <c r="E66">
+        <v>-0.4746550901101985</v>
+      </c>
+      <c r="F66">
+        <v>0.6353833601244647</v>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>ssid_control</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>overall mean</t>
+        </is>
+      </c>
+      <c r="B67">
+        <v>0.2997854549076612</v>
+      </c>
+      <c r="C67">
+        <v>0.007061666277166398</v>
+      </c>
+      <c r="D67">
+        <v>445.5907278586985</v>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>ssid_heat</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>treatment CH</t>
+        </is>
+      </c>
+      <c r="B68">
+        <v>0.00681730462960672</v>
+      </c>
+      <c r="C68">
+        <v>0.005983753811563602</v>
+      </c>
+      <c r="D68">
+        <v>445.5907278586985</v>
+      </c>
+      <c r="E68">
+        <v>1.139302324977388</v>
+      </c>
+      <c r="F68">
+        <v>0.2551891689127502</v>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>ssid_heat</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>treatment LH</t>
+        </is>
+      </c>
+      <c r="B69">
+        <v>-0.00681730462960672</v>
+      </c>
+      <c r="C69">
+        <v>0.005983753811563602</v>
+      </c>
+      <c r="D69">
+        <v>445.5907278586985</v>
+      </c>
+      <c r="E69">
+        <v>-1.139302324977388</v>
+      </c>
+      <c r="F69">
+        <v>0.2551891689127502</v>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>ssid_heat</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>site Emerald</t>
+        </is>
+      </c>
+      <c r="B70">
+        <v>0.0009454295200049829</v>
+      </c>
+      <c r="C70">
+        <v>0.01381901904423573</v>
+      </c>
+      <c r="D70">
+        <v>445.5907278586985</v>
+      </c>
+      <c r="E70">
+        <v>0.06841509639566967</v>
+      </c>
+      <c r="F70">
+        <v>0.9454858939566231</v>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>ssid_heat</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>site Rainbow</t>
+        </is>
+      </c>
+      <c r="B71">
+        <v>-0.006492578208423886</v>
+      </c>
+      <c r="C71">
+        <v>0.01439500216888586</v>
+      </c>
+      <c r="D71">
+        <v>445.5907278586985</v>
+      </c>
+      <c r="E71">
+        <v>-0.4510300264113399</v>
+      </c>
+      <c r="F71">
+        <v>0.6521873154217532</v>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>ssid_heat</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>site Star</t>
+        </is>
+      </c>
+      <c r="B72">
+        <v>-0.005120783672600618</v>
+      </c>
+      <c r="C72">
+        <v>0.008315175380848944</v>
+      </c>
+      <c r="D72">
+        <v>445.5907278586985</v>
+      </c>
+      <c r="E72">
+        <v>-0.6158359190347958</v>
+      </c>
+      <c r="F72">
+        <v>0.5383172526093408</v>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>ssid_heat</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>site MacN</t>
+        </is>
+      </c>
+      <c r="B73">
+        <v>0.01066793236101926</v>
+      </c>
+      <c r="C73">
+        <v>0.01025825578977483</v>
+      </c>
+      <c r="D73">
+        <v>445.5907278586985</v>
+      </c>
+      <c r="E73">
+        <v>1.039936279582031</v>
+      </c>
+      <c r="F73">
+        <v>0.2989334455417383</v>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>ssid_heat</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>treatment x site CH : Emerald</t>
+        </is>
+      </c>
+      <c r="B74">
+        <v>-0.0112139561636805</v>
+      </c>
+      <c r="C74">
+        <v>0.008079237944350287</v>
+      </c>
+      <c r="D74">
+        <v>445.5907278586985</v>
+      </c>
+      <c r="E74">
+        <v>-1.38799676911636</v>
+      </c>
+      <c r="F74">
+        <v>0.1658316239187297</v>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>ssid_heat</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>treatment x site LH : Emerald</t>
+        </is>
+      </c>
+      <c r="B75">
+        <v>0.0112139561636805</v>
+      </c>
+      <c r="C75">
+        <v>0.008079237944350287</v>
+      </c>
+      <c r="D75">
+        <v>445.5907278586985</v>
+      </c>
+      <c r="E75">
+        <v>1.38799676911636</v>
+      </c>
+      <c r="F75">
+        <v>0.1658316239187297</v>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>ssid_heat</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>treatment x site CH : Rainbow</t>
+        </is>
+      </c>
+      <c r="B76">
+        <v>0.0007301870897695557</v>
+      </c>
+      <c r="C76">
+        <v>0.008175471303330168</v>
+      </c>
+      <c r="D76">
+        <v>445.5907278586985</v>
+      </c>
+      <c r="E76">
+        <v>0.08931437255147893</v>
+      </c>
+      <c r="F76">
+        <v>0.9288722013095607</v>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>ssid_heat</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>treatment x site LH : Rainbow</t>
+        </is>
+      </c>
+      <c r="B77">
+        <v>-0.0007301870897695557</v>
+      </c>
+      <c r="C77">
+        <v>0.008175471303330168</v>
+      </c>
+      <c r="D77">
+        <v>445.5907278586985</v>
+      </c>
+      <c r="E77">
+        <v>-0.08931437255147893</v>
+      </c>
+      <c r="F77">
+        <v>0.9288722013095607</v>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>ssid_heat</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>treatment x site CH : Star</t>
+        </is>
+      </c>
+      <c r="B78">
+        <v>0.002999498040475423</v>
+      </c>
+      <c r="C78">
+        <v>0.007972202743448469</v>
+      </c>
+      <c r="D78">
+        <v>445.5907278586985</v>
+      </c>
+      <c r="E78">
+        <v>0.3762445759348508</v>
+      </c>
+      <c r="F78">
+        <v>0.706914154744372</v>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>ssid_heat</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>treatment x site LH : Star</t>
+        </is>
+      </c>
+      <c r="B79">
+        <v>-0.002999498040475423</v>
+      </c>
+      <c r="C79">
+        <v>0.007972202743448469</v>
+      </c>
+      <c r="D79">
+        <v>445.5907278586985</v>
+      </c>
+      <c r="E79">
+        <v>-0.3762445759348508</v>
+      </c>
+      <c r="F79">
+        <v>0.706914154744372</v>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>ssid_heat</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>treatment x site CH : MacN</t>
+        </is>
+      </c>
+      <c r="B80">
+        <v>0.00748427103343552</v>
+      </c>
+      <c r="C80">
+        <v>0.008097573027617034</v>
+      </c>
+      <c r="D80">
+        <v>445.5907278586985</v>
+      </c>
+      <c r="E80">
+        <v>0.9242610110350561</v>
+      </c>
+      <c r="F80">
+        <v>0.3558506772991563</v>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>ssid_heat</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>treatment x site LH : MacN</t>
+        </is>
+      </c>
+      <c r="B81">
+        <v>-0.00748427103343552</v>
+      </c>
+      <c r="C81">
+        <v>0.008097573027617034</v>
+      </c>
+      <c r="D81">
+        <v>445.5907278586985</v>
+      </c>
+      <c r="E81">
+        <v>-0.9242610110350561</v>
+      </c>
+      <c r="F81">
+        <v>0.3558506772991563</v>
+      </c>
+      <c r="G81" t="inlineStr">
         <is>
           <t>ssid_heat</t>
         </is>
@@ -2079,7 +3548,7 @@
         <v>1.099842046264552</v>
       </c>
       <c r="E2">
-        <v>0.9525</v>
+        <v>0.9675</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2139,7 +3608,7 @@
         <v>1.099842046264552</v>
       </c>
       <c r="E5">
-        <v>0.9399999999999999</v>
+        <v>0.9375</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -2163,7 +3632,7 @@
         <v>1.028380681908756</v>
       </c>
       <c r="E6">
-        <v>0.765</v>
+        <v>0.755</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -2223,7 +3692,7 @@
         <v>1.028380681908756</v>
       </c>
       <c r="E9">
-        <v>0.72</v>
+        <v>0.75</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -2247,7 +3716,7 @@
         <v>0.9846049942494004</v>
       </c>
       <c r="E10">
-        <v>0.35</v>
+        <v>0.3525</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -2307,7 +3776,7 @@
         <v>0.9846049942494004</v>
       </c>
       <c r="E13">
-        <v>0.4</v>
+        <v>0.3625</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -2331,7 +3800,7 @@
         <v>1.0879677294264</v>
       </c>
       <c r="E14">
-        <v>0.985</v>
+        <v>0.9925</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -2391,7 +3860,7 @@
         <v>1.0879677294264</v>
       </c>
       <c r="E17">
-        <v>0.9975000000000001</v>
+        <v>1</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>

</xml_diff>